<commit_message>
Tambah sistem jadwal otomatis SMKPD AI
</commit_message>
<xml_diff>
--- a/smkpd-ai-web/public/templates/items/PENGGUNA.xlsx
+++ b/smkpd-ai-web/public/templates/items/PENGGUNA.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PETUNJUK" sheetId="1" r:id="R10b4502900e2494c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DATA" sheetId="2" r:id="Rf3fe7db818e94965"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PETUNJUK" sheetId="1" r:id="R024e2b699a3a4c29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DATA" sheetId="2" r:id="R6aa712e4837b43ae"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -285,12 +285,12 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="65" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="70" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="12" t="str">
-        <x:v>TEMPLATE IMPORT PENGGUNA</x:v>
+        <x:v>TEMPLATE PENGGUNA — SMKPD AI</x:v>
       </x:c>
       <x:c r="B1" s="12"/>
       <x:c r="C1" s="4"/>
@@ -300,42 +300,42 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="13" t="str">
-        <x:v>Jenis Data</x:v>
+        <x:v>Cara</x:v>
       </x:c>
       <x:c r="B2" s="14" t="str">
-        <x:v>PENGGUNA</x:v>
+        <x:v>Isi sheet DATA dan import melalui Database &amp; Excel.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="13" t="str">
-        <x:v>Cara Penggunaan</x:v>
+        <x:v>Satu Jenis Data</x:v>
       </x:c>
       <x:c r="B3" s="14" t="str">
-        <x:v>Isi hanya data pada sheet DATA, lalu unggah melalui menu Database &amp; Excel.</x:v>
+        <x:v>Gunakan satu file untuk satu item agar mudah diperiksa.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="13" t="str">
-        <x:v>Satu Proses</x:v>
+        <x:v>Catatan</x:v>
       </x:c>
       <x:c r="B4" s="14" t="str">
-        <x:v>Satu file digunakan untuk satu jenis data agar pemeriksaan dan perbaikan lebih mudah.</x:v>
+        <x:v>Role tersedia: Admin, Kepala Sekolah, Waka Kurikulum, Guru, Taruna, dan Wali Taruna.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="13" t="str">
-        <x:v>Kunci Unik</x:v>
+        <x:v>Ukuran</x:v>
       </x:c>
       <x:c r="B5" s="14" t="str">
-        <x:v>username</x:v>
+        <x:v>Maksimal 30 MB per file.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="13" t="str">
-        <x:v>Catatan</x:v>
+        <x:v>Kode</x:v>
       </x:c>
       <x:c r="B6" s="14" t="str">
-        <x:v>Role: Admin, Kepala Sekolah, Guru, Taruna, Wali Taruna. Username harus unik.</x:v>
+        <x:v>Gunakan kode singkat dan konsisten.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -349,14 +349,6 @@
     <x:row r="8">
       <x:c r="A8" s="14"/>
       <x:c r="B8" s="14"/>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="14"/>
-      <x:c r="B9" s="14"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="14"/>
-      <x:c r="B10" s="14"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -374,7 +366,7 @@
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -409,7 +401,7 @@
         <x:v>password123</x:v>
       </x:c>
       <x:c r="D2" s="28" t="str">
-        <x:v>Guru</x:v>
+        <x:v>Waka Kurikulum</x:v>
       </x:c>
       <x:c r="E2" s="28" t="str"/>
       <x:c r="F2" s="28" t="str">
@@ -8402,11 +8394,11 @@
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="D2:D1000">
+      <x:formula1>"Admin,Kepala Sekolah,Waka Kurikulum,Guru,Taruna,Wali Taruna"</x:formula1>
+    </x:dataValidation>
     <x:dataValidation type="list" sqref="F2:F1000">
       <x:formula1>"Aktif,Nonaktif"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="D2:D1000">
-      <x:formula1>"Admin,Kepala Sekolah,Guru,Taruna,Wali Taruna"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>